<commit_message>
Add automatic door power wiring sheet to import workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016xNaUwbPDwzomNikmNj8Xy
</commit_message>
<xml_diff>
--- a/本願寺_自動ドアスロープ_取込用.xlsx
+++ b/本願寺_自動ドアスロープ_取込用.xlsx
@@ -10,7 +10,8 @@
     <sheet name="仮設スロープ工事" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="スロープ工事" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="外壁工事" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="確認用（取込しない）" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="自動ドア電源工事" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="確認用（取込しない）" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -548,7 +549,6 @@
           <t>仮設スロープ設置</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
         <v>1</v>
       </c>
@@ -701,7 +701,6 @@
           <t>石畳解体</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
         <v>2</v>
       </c>
@@ -726,7 +725,6 @@
           <t>腰石解体</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="n">
         <v>1</v>
       </c>
@@ -751,7 +749,6 @@
           <t>スロープ工事</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
         <v>4</v>
       </c>
@@ -935,7 +932,6 @@
           <t>サッシ解体</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
         <v>2</v>
       </c>
@@ -960,7 +956,6 @@
           <t>外壁解体</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="n">
         <v>1</v>
       </c>
@@ -985,7 +980,6 @@
           <t>外壁もどし</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
         <v>4</v>
       </c>
@@ -1010,7 +1004,6 @@
           <t>内壁もどし</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="n">
         <v>4</v>
       </c>
@@ -1252,7 +1245,6 @@
           <t>グラスウール</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="n">
         <v>6</v>
       </c>
@@ -1284,7 +1276,286 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>品名</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>仕様</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>見積数量</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>見積単位</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>見積単価</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>原価数量</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>原価単位</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>原価単価</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>分電盤 分岐ブレーカー増設</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>自動ドア専用回路 2P1E 20A</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>箇所</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>8000</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>箇所</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>電源配線</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>VVF2.0-2C 隠ぺい配線</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>20</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F3" t="n">
+        <v>20</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>配管</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PF管16 露出・保護部</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>800</v>
+      </c>
+      <c r="F4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>自動ドア用電源スイッチ取付</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>点検用 手元開閉器</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>箇所</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>6000</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>箇所</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>制御盤結線・試運転立会い</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>自動ドアエンジン一次側</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>式</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>式</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>貫通・開口・補修</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>壁・天井 配線ルート</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>式</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>10000</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>式</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>雑材・運搬費</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>式</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>8000</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>式</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1371,16 +1642,31 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>自動ドア電源工事</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>7</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>見積金額計 79,000円（原価は電気屋さん見積待ち）</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>23</v>
-      </c>
-      <c r="C5" s="2" t="n">
+      <c r="B6">
+        <f>SUM(B2:B5)</f>
+        <v/>
+      </c>
+      <c r="C6" s="2" t="n">
         <v>147160</v>
       </c>
-      <c r="D5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add interior and exterior finishing sheets to import workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016xNaUwbPDwzomNikmNj8Xy
</commit_message>
<xml_diff>
--- a/本願寺_自動ドアスロープ_取込用.xlsx
+++ b/本願寺_自動ドアスロープ_取込用.xlsx
@@ -11,7 +11,9 @@
     <sheet name="スロープ工事" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="外壁工事" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="自動ドア電源工事" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="確認用（取込しない）" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="内装仕上げ工事" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="外装仕上げ工事" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="確認用（取込しない）" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1523,7 +1525,6 @@
           <t>雑材・運搬費</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="n">
         <v>1</v>
       </c>
@@ -1555,7 +1556,596 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>品名</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>仕様</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>見積数量</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>見積単位</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>見積単価</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>原価数量</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>原価単位</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>原価単価</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PB継目・ビス穴 パテ処理</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>自動ドア両袖 壁 (4.5m-3.54m)×H2.47m</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>㎡</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>㎡</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ビニルクロス貼り</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>量産品 既存近似色</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>㎡</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>㎡</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>既存クロス取合い補修</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>式</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>8000</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>式</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ソフト巾木</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>H60 スロープ脇</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>既存カーペット撤去・処分</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>㎡</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F6" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>㎡</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>カーペット張替え</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>自動ドア内側 床</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>㎡</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>7000</v>
+      </c>
+      <c r="F7" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>㎡</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ドア枠廻りシーリング</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>内部側 変成シリコン</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>800</v>
+      </c>
+      <c r="F8" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>小工事割増</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>内装 少量施工</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>式</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>式</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>品名</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>仕様</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>見積数量</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>見積単位</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>見積単価</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>原価数量</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>原価単位</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>原価単価</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>透湿防水シート張り</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>自動ドア両袖 外壁 (4.5m-3.54m)×H2.47m</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>㎡</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>800</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>㎡</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ラス張り</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>波形ラス</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>㎡</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>㎡</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>モルタル塗り</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>下塗り・中塗り 既存取合い共</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>㎡</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>6000</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>㎡</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>外壁仕上げ塗装</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>吹付 既存近似色</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>㎡</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>3500</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>㎡</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>土台水切り</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ガルバリウム鋼板</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ドア枠廻りシーリング</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>外部側 変成シリコン</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F7" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>小工事割増</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>左官・塗装 少量施工</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>式</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>30000</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>式</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1657,14 +2247,44 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>内装仕上げ工事</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>見積金額計 93,600円</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>外装仕上げ工事</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>7</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>見積金額計 72,720円</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="B6">
-        <f>SUM(B2:B5)</f>
+      <c r="B8">
+        <f>SUM(B2:B7)</f>
         <v/>
       </c>
-      <c r="C6" s="2" t="n">
+      <c r="C8" s="2" t="n">
         <v>147160</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add exterior works (外構) sheet to import workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016xNaUwbPDwzomNikmNj8Xy
</commit_message>
<xml_diff>
--- a/本願寺_自動ドアスロープ_取込用.xlsx
+++ b/本願寺_自動ドアスロープ_取込用.xlsx
@@ -13,7 +13,8 @@
     <sheet name="自動ドア電源工事" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="内装仕上げ工事" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="外装仕上げ工事" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="確認用（取込しない）" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="外構工事" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="確認用（取込しない）" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1679,7 +1680,6 @@
           <t>既存クロス取合い補修</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
         <v>1</v>
       </c>
@@ -1737,7 +1737,6 @@
           <t>既存カーペット撤去・処分</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="n">
         <v>6.8</v>
       </c>
@@ -2145,7 +2144,530 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:H16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>品名</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>仕様</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>見積数量</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>見積単位</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>見積単価</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>原価数量</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>原価単位</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>原価単価</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>土間コンクリート打設</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>t100 ワイヤーメッシュ・砕石共 金ゴテ仕上</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>㎡</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>12000</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>㎡</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>石畳 石材</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>900×300×50 既存近似</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>枚</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>18000</v>
+      </c>
+      <c r="F3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>枚</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>石畳 石材</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>600×300×50 既存近似</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>枚</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>12000</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>枚</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>石材据付・目地</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>石工 モルタル敷き 加工共</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>人工</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>35000</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>人工</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>U字溝据付</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>U字溝100</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>9000</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>グレーチング</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>100用 歩行用 細目</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>12000</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>集水桝新設</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>400×400×500 据付共</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>箇所</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>45000</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>箇所</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>集水桝蓋</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>グレーチング 400角</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>枚</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>枚</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>排水管接続</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>既存排水管（管天-220）へ接続</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>式</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>20000</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>式</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>基礎巾木 石材</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>W845×H600×D40</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>枚</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>38000</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>枚</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>基礎巾木 石材取替</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>既存撤去・据付</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>式</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>20000</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>式</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>雨樋一部撤去</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>式</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>式</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>竪樋新設・接続</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>φ60 受金物・継手共</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>3500</v>
+      </c>
+      <c r="F14" t="n">
+        <v>3</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ガラ・残土処分</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>運搬費共</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>式</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>30000</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>式</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>小運搬・養生</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>式</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>10000</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>式</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2277,14 +2799,29 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>外構工事</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>15</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>見積金額計 379,200円</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="B8">
-        <f>SUM(B2:B7)</f>
+      <c r="B9">
+        <f>SUM(B2:B8)</f>
         <v/>
       </c>
-      <c r="C8" s="2" t="n">
+      <c r="C9" s="2" t="n">
         <v>147160</v>
       </c>
     </row>

</xml_diff>